<commit_message>
Update Disc catalog Excel file with new data
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Disc_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Disc_katalog_full.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="BuÇalışmaKitabı" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\Repxpert\src\data\katalogInfo\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88731EF8-DCFB-4789-98E9-5802B9C318F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7B1BE2-CAB0-4489-B8EA-8675AB850701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8616" uniqueCount="8153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8617" uniqueCount="8155">
   <si>
     <t>BREMBO</t>
   </si>
@@ -24495,13 +24495,19 @@
   </si>
   <si>
     <t>KAWE-61162 10</t>
+  </si>
+  <si>
+    <t>78BD0570-2</t>
+  </si>
+  <si>
+    <t>92237703</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -24521,6 +24527,15 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="162"/>
@@ -24559,7 +24574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -24618,6 +24633,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -33716,6 +33735,9 @@
       <c r="B259" s="10" t="s">
         <v>2129</v>
       </c>
+      <c r="C259" s="21" t="s">
+        <v>8153</v>
+      </c>
       <c r="E259" s="2" t="s">
         <v>2130</v>
       </c>
@@ -47660,8 +47682,8 @@
       <c r="B649" s="10" t="s">
         <v>5484</v>
       </c>
-      <c r="D649" s="10" t="s">
-        <v>5484</v>
+      <c r="D649" s="22" t="s">
+        <v>8154</v>
       </c>
       <c r="E649" s="2" t="s">
         <v>5485</v>
@@ -56626,7 +56648,7 @@
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" style="20" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" style="20" customWidth="1"/>
     <col min="3" max="3" width="39.88671875" style="13" customWidth="1"/>
     <col min="4" max="16384" width="8.88671875" style="13"/>
   </cols>

</xml_diff>

<commit_message>
feat: Update Excel files for vehicle compatibility and catalog information
</commit_message>
<xml_diff>
--- a/src/resources/data/catalogInfo/excels/Disc_katalog_full.xlsx
+++ b/src/resources/data/catalogInfo/excels/Disc_katalog_full.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\URETIM9\Desktop\Projects\API_SCRAPE\src\resources\data\catalogInfo\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7B1BE2-CAB0-4489-B8EA-8675AB850701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2446C3-7CB9-497D-A66B-977B1D71E72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2196" yWindow="2196" windowWidth="20532" windowHeight="10140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="BULUNAMAYANLAR" sheetId="7" r:id="rId2"/>
+    <sheet name="API BULUNAMAYANLAR" sheetId="8" r:id="rId2"/>
+    <sheet name="BULUNAMAYANLAR" sheetId="7" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">BULUNAMAYANLAR!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">BULUNAMAYANLAR!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$CM$1090</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8617" uniqueCount="8155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8677" uniqueCount="8155">
   <si>
     <t>BREMBO</t>
   </si>
@@ -56642,6 +56643,771 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB94B13C-9445-4D8C-AF53-C8032F38560D}">
+  <dimension ref="A1:A151"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>7349</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>13001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>13003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>18068</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>19039</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>28052</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>24173</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>43188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>60206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>53229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>34234</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>53228</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>34233</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>25240</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>59239</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>33247</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>49113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>43302</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>49306</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>45340</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>28341</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>25236</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>59354</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>40369</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>43398</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>43399</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>65413</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>63417</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>63418</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>43464</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>40157</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>32472</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>37479</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>68468</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>45488</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>18489</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37491</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>67517</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>25512</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>69556</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>69549</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>27093</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>13577</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>69592</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>40748</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>25730</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>37787</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>25901</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>40903</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>40904</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>25905</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>25906</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>25909</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>25910</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>24916</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>6802</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>6804</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>6806</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>6812</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>6818</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>6826</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>6830</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>6831</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>6833</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>6835</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>6837</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>6839</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>6842</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>6844</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>6846</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>6847</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>6849</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>6851</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>6853</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>6855</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>6857</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>6873</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>6876</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>6968</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>63998</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>6977</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>6980</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>6982</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>6984</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>6987</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>6990</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>6991</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>6993</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>6995</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>6997</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>7001</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>161062</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>161063</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>7017</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>201076</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>201077</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>601078</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>601079</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>7070</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>7071</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102">
+        <v>631511</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>7076</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>7079</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>431512</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>69898</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>281060</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108">
+        <v>401530</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109">
+        <v>691529</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110">
+        <v>341532</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <v>261533</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>7202</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>151536</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>301538</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>401539</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>251540</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>151544</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>681546</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <v>681547</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>761548</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>761549</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A122">
+        <v>681550</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A123">
+        <v>681551</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A124">
+        <v>131553</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A125">
+        <v>131554</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>7263</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A127">
+        <v>721556</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A128">
+        <v>721557</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A129">
+        <v>681560</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A130">
+        <v>681561</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A131">
+        <v>401568</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>7293</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>7294</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>7295</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>7296</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>7297</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>7298</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>7299</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>7300</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>7301</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>7302</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>7303</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>7305</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>7307</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>7309</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>7311</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>7313</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A148">
+        <v>681569</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A149">
+        <v>531571</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A150">
+        <v>531572</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A151">
+        <v>511577</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF5782AC-442B-4F17-B228-00366512F92C}">
   <sheetPr codeName="Sayfa3"/>
   <dimension ref="A1:C154"/>

</xml_diff>